<commit_message>
Écarter les lignes hors matière du calcul d'écart et fiabiliser les livrables
Le rapport annonçait 51 « PLU sans fiche technique » alors que 3 lignes du PMIX
ne consomment aucune matière (50000 GLOVO, 8017 ENFT JOUET, 5505 NO Sauce) :
leur demander une fiche était une fausse anomalie. Elles sont désormais listées
à part, hors du calcul théorique, dans le rapport et la feuille Anomalies.

Colonne « CA FCFA » des menus PMIX renommée « Coût théorique (F) » : la valeur
affichée est le coût de fiche, jamais une recette, ce qui rendait la libellé
trompeur.

Noms du référentiel PMIX (missingPmix.js) recalés PLU par PLU sur la fiche
technique transmise par le CDG le 21/10 — la liste d'origine était décalée d'une
ligne sur 192 entrées.

Ajout du déploiement serveur (docker-compose.yml, .env.production.example sans
secrets réels) et du script de re-dérivation des prix backend.
</commit_message>
<xml_diff>
--- a/frontend/public/exemple inventaire.xlsx
+++ b/frontend/public/exemple inventaire.xlsx
@@ -6449,172 +6449,98 @@
       <c r="R45" s="56"/>
     </row>
     <row r="46" spans="2:18" s="24" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B46" s="57" t="s">
-        <v>23</v>
-      </c>
-      <c r="C46" s="58" t="s">
-        <v>24</v>
-      </c>
-      <c r="D46" s="59" t="s">
-        <v>111</v>
-      </c>
-      <c r="E46" s="73">
-        <v>25</v>
-      </c>
+      <c r="B46" s="57"/>
+      <c r="C46" s="58"/>
+      <c r="D46" s="59"/>
+      <c r="E46" s="73"/>
       <c r="F46" s="61"/>
       <c r="G46" s="67"/>
       <c r="H46" s="67"/>
-      <c r="I46" s="64">
-        <v>0</v>
-      </c>
+      <c r="I46" s="64"/>
       <c r="J46" s="65">
         <f>I46</f>
-        <v>0</v>
-      </c>
-      <c r="K46" s="68" t="s">
-        <v>100</v>
-      </c>
+      </c>
+      <c r="K46" s="68"/>
       <c r="L46" s="51"/>
       <c r="M46" s="52">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="N46" s="53"/>
-      <c r="O46" s="54">
-        <v>5410033853002</v>
-      </c>
+      <c r="O46" s="54"/>
       <c r="P46" s="55">
         <f>I46+G46*E46</f>
-        <v>0</v>
       </c>
       <c r="R46" s="56"/>
     </row>
     <row r="47" spans="2:18" s="24" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B47" s="57" t="s">
-        <v>23</v>
-      </c>
-      <c r="C47" s="58" t="s">
-        <v>24</v>
-      </c>
-      <c r="D47" s="59" t="s">
-        <v>112</v>
-      </c>
-      <c r="E47" s="60">
-        <v>12</v>
-      </c>
+      <c r="B47" s="57"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="59"/>
+      <c r="E47" s="60"/>
       <c r="F47" s="61"/>
-      <c r="G47" s="62">
-        <v>0</v>
-      </c>
+      <c r="G47" s="62"/>
       <c r="H47" s="67"/>
-      <c r="I47" s="64">
-        <v>0</v>
-      </c>
+      <c r="I47" s="64"/>
       <c r="J47" s="65">
         <f>G47+I47/E47</f>
-        <v>0</v>
-      </c>
-      <c r="K47" s="68" t="s">
-        <v>113</v>
-      </c>
+      </c>
+      <c r="K47" s="68"/>
       <c r="L47" s="51"/>
       <c r="M47" s="52">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="N47" s="53"/>
-      <c r="O47" s="54">
-        <v>4033854001301</v>
-      </c>
+      <c r="O47" s="54"/>
       <c r="P47" s="55">
         <f t="shared" si="7"/>
-        <v>0</v>
       </c>
       <c r="R47" s="56"/>
     </row>
     <row r="48" spans="2:18" s="24" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B48" s="41" t="s">
-        <v>23</v>
-      </c>
-      <c r="C48" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="D48" s="69" t="s">
-        <v>114</v>
-      </c>
-      <c r="E48" s="70">
-        <v>12</v>
-      </c>
+      <c r="B48" s="41"/>
+      <c r="C48" s="42"/>
+      <c r="D48" s="69"/>
+      <c r="E48" s="70"/>
       <c r="F48" s="71"/>
-      <c r="G48" s="62">
-        <v>0</v>
-      </c>
+      <c r="G48" s="62"/>
       <c r="H48" s="67"/>
-      <c r="I48" s="64">
-        <v>0</v>
-      </c>
+      <c r="I48" s="64"/>
       <c r="J48" s="49">
         <f>G48+I48/E48</f>
-        <v>0</v>
-      </c>
-      <c r="K48" s="68" t="s">
-        <v>113</v>
-      </c>
+      </c>
+      <c r="K48" s="68"/>
       <c r="L48" s="51"/>
       <c r="M48" s="52">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="N48" s="53"/>
-      <c r="O48" s="54" t="s">
-        <v>115</v>
-      </c>
+      <c r="O48" s="54"/>
       <c r="P48" s="55">
         <f t="shared" si="7"/>
-        <v>0</v>
       </c>
       <c r="R48" s="56"/>
     </row>
     <row r="49" spans="2:19" s="24" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B49" s="41" t="s">
-        <v>23</v>
-      </c>
-      <c r="C49" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="D49" s="69" t="s">
-        <v>116</v>
-      </c>
-      <c r="E49" s="70">
-        <v>6</v>
-      </c>
+      <c r="B49" s="41"/>
+      <c r="C49" s="42"/>
+      <c r="D49" s="69"/>
+      <c r="E49" s="70"/>
       <c r="F49" s="71"/>
-      <c r="G49" s="62">
-        <v>0</v>
-      </c>
+      <c r="G49" s="62"/>
       <c r="H49" s="67"/>
-      <c r="I49" s="64">
-        <v>0</v>
-      </c>
+      <c r="I49" s="64"/>
       <c r="J49" s="49">
         <f>G49+I49/E49</f>
-        <v>0</v>
-      </c>
-      <c r="K49" s="68" t="s">
-        <v>117</v>
-      </c>
+      </c>
+      <c r="K49" s="68"/>
       <c r="L49" s="51"/>
       <c r="M49" s="52">
         <f t="shared" si="1"/>
-        <v>0</v>
       </c>
       <c r="N49" s="53"/>
-      <c r="O49" s="54" t="s">
-        <v>118</v>
-      </c>
+      <c r="O49" s="54"/>
       <c r="P49" s="55">
         <f>I49+G49*E49</f>
-        <v>0</v>
       </c>
       <c r="R49" s="56"/>
     </row>

</xml_diff>